<commit_message>
Fix Gerente name not showing, stray "Otros" line, and a stray orange cell
- GERENTE_PROYECTO now resolves the Gerente's real name via
  get_connected_person() instead of reading .text off the Connect
  Boards column directly, which wasn't reliably populated - same fix
  already proven for the Gerente's email.
- build_services() now excludes the literal "Otros" option text from
  the rendered list, matching build_template_points()'s existing
  behavior - previously it showed both "Otros" and the actual custom
  text typed in "Especifique Otro Servicio".
- Template: K62/M62 (Dias/Observaciones, first row of Programacion de
  Fechas) had a stray orange font color left over from an earlier edit;
  matched to the black theme color used everywhere else in that table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -1303,7 +1303,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="296">
+  <cellXfs count="298">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2242,6 +2242,12 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="9" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="67" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4379,9 +4385,9 @@
       <c r="H62" s="129" t="n"/>
       <c r="I62" s="243" t="n"/>
       <c r="J62" s="244" t="n"/>
-      <c r="K62" s="279" t="n"/>
+      <c r="K62" s="296" t="n"/>
       <c r="L62" s="280" t="n"/>
-      <c r="M62" s="189" t="n"/>
+      <c r="M62" s="297" t="n"/>
       <c r="N62" s="187" t="n"/>
       <c r="O62" s="187" t="n"/>
       <c r="P62" s="188" t="n"/>

</xml_diff>

<commit_message>
Match Puntos de Revision title width to its table, unify Servicios Basicos header color
- E83:P83 -> E83:M83: the title now spans the same width as the actual
  table below it (E:M), instead of stretching wider to P and looking
  off-center relative to the data.
- Servicios Basicos header (D75/E75) now uses the same solid-orange
  fill with white text as every other section header, instead of the
  light-background/orange-text style it had.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -1303,7 +1303,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="298">
+  <cellXfs count="300">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2248,6 +2248,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="29" fillId="4" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4648,12 +4654,12 @@
     <row r="75" ht="24.9" customHeight="1">
       <c r="B75" s="74" t="n"/>
       <c r="C75" s="74" t="n"/>
-      <c r="D75" s="288" t="inlineStr">
+      <c r="D75" s="298" t="inlineStr">
         <is>
           <t>NO.</t>
         </is>
       </c>
-      <c r="E75" s="289" t="inlineStr">
+      <c r="E75" s="299" t="inlineStr">
         <is>
           <t>SERVICIOS BASICOS NECESARIOS PARA TRABAJAR</t>
         </is>
@@ -5757,7 +5763,6 @@
     <mergeCell ref="D45:I45"/>
     <mergeCell ref="D23:H23"/>
     <mergeCell ref="L38:O38"/>
-    <mergeCell ref="E83:P83"/>
     <mergeCell ref="E51:J51"/>
     <mergeCell ref="L31:O31"/>
     <mergeCell ref="L40:O40"/>
@@ -5807,6 +5812,7 @@
     <mergeCell ref="I19:J19"/>
     <mergeCell ref="D48:P48"/>
     <mergeCell ref="K66:L66"/>
+    <mergeCell ref="E83:M83"/>
     <mergeCell ref="E92:M92"/>
     <mergeCell ref="L20:O20"/>
     <mergeCell ref="F14:J14"/>

</xml_diff>

<commit_message>
Fix inconsistent bold/font-size on the first rows of all three list sections
Puntos de Revision rows 84-85, Trabajos Previos rows 69-70, and
Servicios Basicos rows 76-78 were bold and/or 14pt while every other row
in their own section was regular 12pt - a leftover template
inconsistency. Matched all of them to the same style used by the rest
of their section.

Also corrected _estimate_row_height()'s default font size from 14 to
12pt to match the template's actual font, now that it's consistent -
the previous mismatch meant row heights were being calculated for a
font size larger than what's actually rendered.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -1303,7 +1303,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="300">
+  <cellXfs count="306">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2253,6 +2253,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4537,7 +4555,7 @@
       <c r="D69" s="108" t="n">
         <v>1</v>
       </c>
-      <c r="E69" s="186" t="inlineStr">
+      <c r="E69" s="302" t="inlineStr">
         <is>
           <t>{{TRABAJOS_PREVIOS}}</t>
         </is>
@@ -4562,7 +4580,7 @@
       <c r="D70" s="110" t="n">
         <v>2</v>
       </c>
-      <c r="E70" s="295" t="n"/>
+      <c r="E70" s="303" t="n"/>
       <c r="F70" s="187" t="n"/>
       <c r="G70" s="187" t="n"/>
       <c r="H70" s="187" t="n"/>
@@ -4684,7 +4702,7 @@
       <c r="D76" s="108" t="n">
         <v>1</v>
       </c>
-      <c r="E76" s="192" t="inlineStr">
+      <c r="E76" s="304" t="inlineStr">
         <is>
           <t>{{SERVICIOS_BASICOS}}</t>
         </is>
@@ -4709,7 +4727,7 @@
       <c r="D77" s="110" t="n">
         <v>2</v>
       </c>
-      <c r="E77" s="197" t="n"/>
+      <c r="E77" s="305" t="n"/>
       <c r="F77" s="187" t="n"/>
       <c r="G77" s="187" t="n"/>
       <c r="H77" s="187" t="n"/>
@@ -4730,7 +4748,7 @@
       <c r="D78" s="108" t="n">
         <v>3</v>
       </c>
-      <c r="E78" s="192" t="n"/>
+      <c r="E78" s="304" t="n"/>
       <c r="F78" s="187" t="n"/>
       <c r="G78" s="187" t="n"/>
       <c r="H78" s="187" t="n"/>
@@ -4841,7 +4859,7 @@
       <c r="D84" s="232" t="n">
         <v>1</v>
       </c>
-      <c r="E84" s="232" t="inlineStr">
+      <c r="E84" s="300" t="inlineStr">
         <is>
           <t>{{PUNTOS_REVISION}}</t>
         </is>
@@ -4866,7 +4884,7 @@
       <c r="D85" s="155" t="n">
         <v>2</v>
       </c>
-      <c r="E85" s="155" t="n"/>
+      <c r="E85" s="301" t="n"/>
       <c r="F85" s="156" t="n"/>
       <c r="G85" s="156" t="n"/>
       <c r="H85" s="156" t="n"/>

</xml_diff>

<commit_message>
Center signature images in their box, uppercase Melissa's printed name
insert_signature() anchored the scaled image at the box's top-left
corner, which only fills one dimension exactly (uniform scaling) -
left visibly off-center whenever the box was wider or taller than the
image. Now computes the leftover space and offsets a OneCellAnchor by
half of it in each direction, so it's centered regardless of the
signature's own aspect ratio. Applies to every signature insertion
(Lider, Gerente, and Melissa all go through this same function).

"Arq. Melissa Alvarenga" under her signature was the only printed name
in the signature block not uppercased (Lider and Gerente already are,
via .upper() in generate_acta.py) - fixed in both template variants.
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="348" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="C-9-12" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hoja1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C-9-12" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="ACOMETIDA">#REF!</definedName>
@@ -2351,7 +2351,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>2</col>
@@ -2369,24 +2369,24 @@
       <nvPicPr>
         <cNvPr id="6" name="Imagen 5"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="555189" y="327972"/>
           <a:ext cx="1806529" cy="1723429"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -2410,24 +2410,24 @@
       <nvPicPr>
         <cNvPr id="7" name="Picture 6"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="12628684" y="363359"/>
           <a:ext cx="2670669" cy="1876779"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -5681,7 +5681,7 @@
       <c r="K123" s="208" t="n"/>
       <c r="L123" s="174" t="inlineStr">
         <is>
-          <t>Arq. Melissa Alvarenga</t>
+          <t>ARQ. MELISSA ALVARENGA</t>
         </is>
       </c>
       <c r="N123" s="208" t="n"/>

</xml_diff>

<commit_message>
Fix DIAS showing "4.00", exclude "Otro" (singular) from Servicios Basicos, and switch the pre-sign status to "Link Enviado"
- _write_programacion() now forces number_format="0" on the DIAS cell
  instead of trusting whatever the template row already had - rows 2
  and 3 of the template had "0.00" baked in, which displayed an
  integer day count as e.g. "4.00". Also fixed those two cells
  directly in both template variants for consistency.
- build_services() only excluded "otros" (plural), but the actual
  Monday multi-select option is "Otro" (singular) - it was never being
  filtered out.
- GERENTE_FIRMA_ESTADO_PENDIENTE changed from "Pendiente" to "Link
  Enviado": the Outlook automation that notifies the Gerente needs a
  status change distinct from anything else on that column to trigger
  on reliably. Requires adding "Link Enviado" as a new option on the
  "Firmado?" status column in Monday and pointing that automation at
  it (done on the Monday side, not here).
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -4431,7 +4431,7 @@
       <c r="H63" s="129" t="n"/>
       <c r="I63" s="253" t="n"/>
       <c r="J63" s="196" t="n"/>
-      <c r="K63" s="202" t="n"/>
+      <c r="K63" s="253" t="n"/>
       <c r="L63" s="196" t="n"/>
       <c r="M63" s="222" t="n"/>
       <c r="N63" s="129" t="n"/>
@@ -4453,7 +4453,7 @@
       <c r="H64" s="129" t="n"/>
       <c r="I64" s="251" t="n"/>
       <c r="J64" s="196" t="n"/>
-      <c r="K64" s="195" t="n"/>
+      <c r="K64" s="251" t="n"/>
       <c r="L64" s="196" t="n"/>
       <c r="M64" s="209" t="n"/>
       <c r="N64" s="129" t="n"/>

</xml_diff>

<commit_message>
Add contract-type note printed at the end of the acta when Melissa signs
Melissa now picks one of three statuses instead of a single generic
FIRMADO: "FIRMADO SIN CONTRATO", "FIRMADO LEGAL", "FIRMADO FASTTRACK".
All three trigger the same signing flow, but each also prints a
different note near the signature block ({{TIPO_CONTRATO_MENSAJE}},
a new placeholder in both template variants) telling Procurement what
to attach when the invoice comes in.

The placeholder is deliberately left out of generate_acta.py's
replacements dict, same as {{FIRMA_MELISSA}} - it has to survive the
Lider/Gerente stages untouched and only gets resolved by
insert_text_placeholder() in sign_document.py once Melissa's chosen
label is known. The old single FIRMA_TRIGGER_LABEL ("FIRMADO") is
retired - the corresponding automation should be deleted in Monday.
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -90,7 +90,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;Q&quot;* #,##0.00_-;\-&quot;Q&quot;* #,##0.00_-;_-&quot;Q&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -301,6 +301,11 @@
       <color theme="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Open Sans"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -1303,7 +1308,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="306">
+  <cellXfs count="307">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2271,6 +2276,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5694,22 +5702,14 @@
       <c r="Q123" s="55" t="n"/>
       <c r="R123" s="55" t="n"/>
     </row>
-    <row r="124" customFormat="1" s="123">
+    <row r="124" ht="27.6" customFormat="1" customHeight="1" s="123">
       <c r="B124" s="74" t="n"/>
       <c r="C124" s="74" t="n"/>
-      <c r="D124" s="55" t="n"/>
-      <c r="E124" s="55" t="n"/>
-      <c r="F124" s="55" t="n"/>
-      <c r="G124" s="55" t="n"/>
-      <c r="H124" s="55" t="n"/>
-      <c r="I124" s="55" t="n"/>
-      <c r="J124" s="55" t="n"/>
-      <c r="K124" s="55" t="n"/>
-      <c r="L124" s="77" t="n"/>
-      <c r="M124" s="77" t="n"/>
-      <c r="N124" s="55" t="n"/>
-      <c r="O124" s="77" t="n"/>
-      <c r="P124" s="78" t="n"/>
+      <c r="D124" s="306" t="inlineStr">
+        <is>
+          <t>{{TIPO_CONTRATO_MENSAJE}}</t>
+        </is>
+      </c>
       <c r="Q124" s="55" t="n"/>
       <c r="R124" s="55" t="n"/>
     </row>
@@ -5737,7 +5737,7 @@
       <c r="R126" s="55" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="197">
+  <mergeCells count="198">
     <mergeCell ref="M61:P61"/>
     <mergeCell ref="H123:J123"/>
     <mergeCell ref="D116:F116"/>
@@ -5816,6 +5816,7 @@
     <mergeCell ref="M64:P64"/>
     <mergeCell ref="G65:H65"/>
     <mergeCell ref="D35:I35"/>
+    <mergeCell ref="D124:P124"/>
     <mergeCell ref="D44:I44"/>
     <mergeCell ref="O123:P123"/>
     <mergeCell ref="D27:J27"/>

</xml_diff>

<commit_message>
Hide the contract-type note placeholder until Melissa signs
{{TIPO_CONTRATO_MENSAJE}} is deliberately left unresolved at generation,
but it was visible in the document the Lider and Gerente review. It now
has white font in both templates (same trick as the signature
placeholders), and insert_text_placeholder switches the font to black
when it writes the real text so the note shows once Melissa signs.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -1308,7 +1308,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="308">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2279,6 +2279,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2746,7 +2749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:W126"/>
+  <dimension ref="A1:W126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="17.4"/>
   <cols>
     <col width="3.109375" customWidth="1" style="148" min="1" max="1"/>
@@ -2771,6 +2774,7 @@
     <col width="11.44140625" customWidth="1" style="148" min="22" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="48" t="n"/>
       <c r="C2" s="48" t="n"/>
@@ -5705,7 +5709,7 @@
     <row r="124" ht="27.6" customFormat="1" customHeight="1" s="123">
       <c r="B124" s="74" t="n"/>
       <c r="C124" s="74" t="n"/>
-      <c r="D124" s="306" t="inlineStr">
+      <c r="D124" s="307" t="inlineStr">
         <is>
           <t>{{TIPO_CONTRATO_MENSAJE}}</t>
         </is>

</xml_diff>

<commit_message>
Polish the Punto de Acta template: spelling, palette, annexes list, tidy page layout
- Templates: accents/typos fixed, softer greys, E4 orange unified, thin grey
  borders in the quotation table, clearer invoice-day text, new ANEXOS block.
- excel_writer: hide empty rows, fit quotation row heights to their text,
  number formats, uniform programacion fonts, recompute page breaks so
  sections are not split and no blank trailing page is printed.
- generate_acta: list the attached cotizacion/documentacion files as anexos.
- acta_builder: AG 229-2014 and 'POR DIA' accent.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
+++ b/templates/100_PUNTO_DE_ACTA_PLANTILLA.xlsx
@@ -79,7 +79,7 @@
     <definedName name="DUCELEC" localSheetId="0">#REF!</definedName>
     <definedName name="ESPECIALES" localSheetId="0">#REF!</definedName>
     <definedName name="EXP" localSheetId="0">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'C-9-12'!$B$2:$R$125</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'C-9-12'!$B$2:$R$136</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -307,7 +307,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -362,8 +362,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEC7828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="85">
+  <borders count="87">
     <border>
       <left/>
       <right/>
@@ -1303,12 +1313,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="308">
+  <cellXfs count="341">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2282,6 +2312,123 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="5" borderId="85" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="85" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="85" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="86" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="48" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="47" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="49" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="64" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="51" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="47" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="47" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="29" fillId="10" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="47" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="13" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="61" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2749,7 +2896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W126"/>
+  <dimension ref="A1:W135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="17.4"/>
   <cols>
     <col width="3.109375" customWidth="1" style="148" min="1" max="1"/>
@@ -3074,7 +3221,7 @@
       <c r="C14" s="59" t="n"/>
       <c r="D14" s="144" t="inlineStr">
         <is>
-          <t>NO. TELEFONO:</t>
+          <t>NO. TELÉFONO:</t>
         </is>
       </c>
       <c r="E14" s="145" t="n"/>
@@ -3144,7 +3291,7 @@
       <c r="C16" s="59" t="n"/>
       <c r="D16" s="268" t="inlineStr">
         <is>
-          <t>NO. COTIZACION</t>
+          <t>NO. COTIZACIÓN</t>
         </is>
       </c>
       <c r="E16" s="269" t="n"/>
@@ -3208,7 +3355,7 @@
       <c r="K18" s="73" t="n"/>
       <c r="L18" s="203" t="inlineStr">
         <is>
-          <t>TIEMPOS DE PAGO CON RECEPCION DE FACTURA</t>
+          <t>TIEMPOS DE PAGO CON RECEPCIÓN DE FACTURA</t>
         </is>
       </c>
       <c r="M18" s="138" t="n"/>
@@ -3248,7 +3395,7 @@
       <c r="O19" s="139" t="n"/>
       <c r="P19" s="84" t="inlineStr">
         <is>
-          <t>15 DIAS</t>
+          <t>15 DÍAS</t>
         </is>
       </c>
       <c r="Q19" s="55" t="n"/>
@@ -3259,7 +3406,7 @@
       <c r="C20" s="74" t="n"/>
       <c r="D20" s="221" t="inlineStr">
         <is>
-          <t>Punto de acta firmado por contratista, genrete E4, lider E4</t>
+          <t>Punto de acta firmado por contratista, gerente E4, líder E4</t>
         </is>
       </c>
       <c r="E20" s="126" t="n"/>
@@ -3283,7 +3430,7 @@
       <c r="O20" s="139" t="n"/>
       <c r="P20" s="85" t="inlineStr">
         <is>
-          <t>30 DIAS</t>
+          <t>30 DÍAS</t>
         </is>
       </c>
       <c r="Q20" s="55" t="n"/>
@@ -3303,7 +3450,7 @@
       <c r="H21" s="127" t="n"/>
       <c r="I21" s="146" t="inlineStr">
         <is>
-          <t>anticipo / estimacion</t>
+          <t>anticipo / estimación</t>
         </is>
       </c>
       <c r="J21" s="126" t="n"/>
@@ -3318,7 +3465,7 @@
       <c r="O21" s="139" t="n"/>
       <c r="P21" s="84" t="inlineStr">
         <is>
-          <t>30 DIAS</t>
+          <t>30 DÍAS</t>
         </is>
       </c>
       <c r="Q21" s="55" t="n"/>
@@ -3373,7 +3520,7 @@
       <c r="H23" s="127" t="n"/>
       <c r="I23" s="146" t="inlineStr">
         <is>
-          <t>para estimacion</t>
+          <t>para estimación</t>
         </is>
       </c>
       <c r="J23" s="126" t="n"/>
@@ -3391,7 +3538,7 @@
       <c r="C24" s="74" t="n"/>
       <c r="D24" s="221" t="inlineStr">
         <is>
-          <t>Carta de garantia</t>
+          <t>Carta de garantía</t>
         </is>
       </c>
       <c r="E24" s="126" t="n"/>
@@ -3446,7 +3593,8 @@
       <c r="O25" s="139" t="n"/>
       <c r="P25" s="84" t="inlineStr">
         <is>
-          <t>Lunes de               8:00 AM- 4:00 PM</t>
+          <t>Lunes de
+8:00 AM a 4:00 PM</t>
         </is>
       </c>
       <c r="Q25" s="55" t="n"/>
@@ -3457,7 +3605,7 @@
       <c r="C26" s="74" t="n"/>
       <c r="D26" s="143" t="inlineStr">
         <is>
-          <t>TODO DOCUMENTO DE ESTIMACION Y ADELANTO DEBE IR FIRMADO POR EL CONTRATISTA</t>
+          <t>TODO DOCUMENTO DE ESTIMACIÓN Y ADELANTO DEBE IR FIRMADO POR EL CONTRATISTA</t>
         </is>
       </c>
       <c r="E26" s="138" t="n"/>
@@ -3477,7 +3625,8 @@
       <c r="O26" s="139" t="n"/>
       <c r="P26" s="85" t="inlineStr">
         <is>
-          <t>Lunes y Martes de 8:00 AM- 4:00 PM</t>
+          <t>Lunes y Martes de
+8:00 AM a 4:00 PM</t>
         </is>
       </c>
       <c r="Q26" s="55" t="n"/>
@@ -3504,7 +3653,8 @@
       <c r="O27" s="139" t="n"/>
       <c r="P27" s="84" t="inlineStr">
         <is>
-          <t>Lunes de               8:00 AM- 4:00 PM</t>
+          <t>Lunes de
+8:00 AM a 4:00 PM</t>
         </is>
       </c>
       <c r="Q27" s="68" t="n"/>
@@ -3584,7 +3734,7 @@
       <c r="O30" s="180" t="n"/>
       <c r="P30" s="9" t="inlineStr">
         <is>
-          <t>1% POR DIA</t>
+          <t>1% POR DÍA</t>
         </is>
       </c>
       <c r="Q30" s="55" t="n"/>
@@ -3665,7 +3815,7 @@
       <c r="C33" s="74" t="n"/>
       <c r="D33" s="124" t="inlineStr">
         <is>
-          <t>Reunión semanal con LIDER DE PROYECTO</t>
+          <t>Reunión semanal con LÍDER DE PROYECTO</t>
         </is>
       </c>
       <c r="E33" s="120" t="n"/>
@@ -3681,7 +3831,7 @@
       <c r="K33" s="55" t="n"/>
       <c r="L33" s="248" t="inlineStr">
         <is>
-          <t>Por no cumplir con documentos de reporteria semanal</t>
+          <t>Por no cumplir con documentos de reportería semanal</t>
         </is>
       </c>
       <c r="M33" s="182" t="n"/>
@@ -3743,7 +3893,7 @@
       <c r="K35" s="55" t="n"/>
       <c r="L35" s="159" t="inlineStr">
         <is>
-          <t>DOCUMENTO ENTREGADOS A CONTRATISTA POR PARTE DE E4</t>
+          <t>DOCUMENTOS ENTREGADOS A CONTRATISTA POR PARTE DE E4</t>
         </is>
       </c>
       <c r="Q35" s="55" t="n"/>
@@ -3792,7 +3942,7 @@
       <c r="K37" s="55" t="n"/>
       <c r="L37" s="221" t="inlineStr">
         <is>
-          <t>Politica de recepcion de facturas y pagos</t>
+          <t>Política de recepción de facturas y pagos</t>
         </is>
       </c>
       <c r="M37" s="126" t="n"/>
@@ -3827,7 +3977,7 @@
       <c r="K38" s="55" t="n"/>
       <c r="L38" s="125" t="inlineStr">
         <is>
-          <t>Politica de SSO en obra</t>
+          <t>Política de SSO en obra</t>
         </is>
       </c>
       <c r="M38" s="126" t="n"/>
@@ -4130,7 +4280,7 @@
       </c>
       <c r="E49" s="154" t="inlineStr">
         <is>
-          <t>DESCRIPCION</t>
+          <t>DESCRIPCIÓN</t>
         </is>
       </c>
       <c r="K49" s="154" t="inlineStr">
@@ -4165,102 +4315,102 @@
     <row r="50" ht="69.90000000000001" customHeight="1">
       <c r="B50" s="8" t="n"/>
       <c r="C50" s="23" t="n"/>
-      <c r="D50" s="293" t="n"/>
-      <c r="E50" s="247" t="n"/>
+      <c r="D50" s="308" t="n"/>
+      <c r="E50" s="309" t="n"/>
       <c r="F50" s="161" t="n"/>
       <c r="G50" s="161" t="n"/>
       <c r="H50" s="161" t="n"/>
       <c r="I50" s="161" t="n"/>
-      <c r="J50" s="133" t="n"/>
+      <c r="J50" s="310" t="n"/>
       <c r="K50" s="26" t="n"/>
-      <c r="L50" s="27" t="n"/>
+      <c r="L50" s="311" t="n"/>
       <c r="M50" s="28" t="n"/>
-      <c r="N50" s="184" t="n"/>
-      <c r="O50" s="133" t="n"/>
+      <c r="N50" s="312" t="n"/>
+      <c r="O50" s="310" t="n"/>
       <c r="P50" s="29" t="n"/>
     </row>
     <row r="51" ht="68.09999999999999" customHeight="1">
       <c r="B51" s="8" t="n"/>
       <c r="C51" s="23" t="n"/>
-      <c r="D51" s="294" t="n"/>
-      <c r="E51" s="178" t="n"/>
+      <c r="D51" s="313" t="n"/>
+      <c r="E51" s="314" t="n"/>
       <c r="F51" s="161" t="n"/>
       <c r="G51" s="161" t="n"/>
       <c r="H51" s="161" t="n"/>
       <c r="I51" s="161" t="n"/>
-      <c r="J51" s="133" t="n"/>
+      <c r="J51" s="310" t="n"/>
       <c r="K51" s="31" t="n"/>
-      <c r="L51" s="32" t="n"/>
+      <c r="L51" s="315" t="n"/>
       <c r="M51" s="33" t="n"/>
-      <c r="N51" s="132" t="n"/>
-      <c r="O51" s="133" t="n"/>
+      <c r="N51" s="316" t="n"/>
+      <c r="O51" s="310" t="n"/>
       <c r="P51" s="34" t="n"/>
     </row>
     <row r="52" ht="68.09999999999999" customHeight="1">
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="23" t="n"/>
-      <c r="D52" s="293" t="n"/>
-      <c r="E52" s="247" t="n"/>
+      <c r="D52" s="308" t="n"/>
+      <c r="E52" s="309" t="n"/>
       <c r="F52" s="161" t="n"/>
       <c r="G52" s="161" t="n"/>
       <c r="H52" s="161" t="n"/>
       <c r="I52" s="161" t="n"/>
-      <c r="J52" s="133" t="n"/>
+      <c r="J52" s="310" t="n"/>
       <c r="K52" s="26" t="n"/>
-      <c r="L52" s="27" t="n"/>
+      <c r="L52" s="311" t="n"/>
       <c r="M52" s="28" t="n"/>
-      <c r="N52" s="184" t="n"/>
-      <c r="O52" s="133" t="n"/>
+      <c r="N52" s="312" t="n"/>
+      <c r="O52" s="310" t="n"/>
       <c r="P52" s="29" t="n"/>
     </row>
     <row r="53" ht="69.90000000000001" customHeight="1">
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="23" t="n"/>
-      <c r="D53" s="294" t="n"/>
-      <c r="E53" s="178" t="n"/>
+      <c r="D53" s="313" t="n"/>
+      <c r="E53" s="314" t="n"/>
       <c r="F53" s="161" t="n"/>
       <c r="G53" s="161" t="n"/>
       <c r="H53" s="161" t="n"/>
       <c r="I53" s="161" t="n"/>
-      <c r="J53" s="133" t="n"/>
+      <c r="J53" s="310" t="n"/>
       <c r="K53" s="31" t="n"/>
-      <c r="L53" s="32" t="n"/>
+      <c r="L53" s="315" t="n"/>
       <c r="M53" s="33" t="n"/>
-      <c r="N53" s="132" t="n"/>
-      <c r="O53" s="133" t="n"/>
+      <c r="N53" s="316" t="n"/>
+      <c r="O53" s="310" t="n"/>
       <c r="P53" s="34" t="n"/>
     </row>
     <row r="54" ht="69.90000000000001" customHeight="1">
       <c r="B54" s="23" t="n"/>
-      <c r="D54" s="293" t="n"/>
-      <c r="E54" s="247" t="n"/>
+      <c r="D54" s="308" t="n"/>
+      <c r="E54" s="309" t="n"/>
       <c r="F54" s="161" t="n"/>
       <c r="G54" s="161" t="n"/>
       <c r="H54" s="161" t="n"/>
       <c r="I54" s="161" t="n"/>
-      <c r="J54" s="133" t="n"/>
+      <c r="J54" s="310" t="n"/>
       <c r="K54" s="26" t="n"/>
-      <c r="L54" s="27" t="n"/>
+      <c r="L54" s="311" t="n"/>
       <c r="M54" s="28" t="n"/>
-      <c r="N54" s="184" t="n"/>
-      <c r="O54" s="133" t="n"/>
+      <c r="N54" s="312" t="n"/>
+      <c r="O54" s="310" t="n"/>
       <c r="P54" s="29" t="n"/>
     </row>
     <row r="55" ht="66.90000000000001" customHeight="1">
       <c r="B55" s="8" t="n"/>
       <c r="C55" s="23" t="n"/>
-      <c r="D55" s="294" t="n"/>
-      <c r="E55" s="178" t="n"/>
+      <c r="D55" s="313" t="n"/>
+      <c r="E55" s="314" t="n"/>
       <c r="F55" s="161" t="n"/>
       <c r="G55" s="161" t="n"/>
       <c r="H55" s="161" t="n"/>
       <c r="I55" s="161" t="n"/>
-      <c r="J55" s="133" t="n"/>
+      <c r="J55" s="310" t="n"/>
       <c r="K55" s="31" t="n"/>
-      <c r="L55" s="32" t="n"/>
+      <c r="L55" s="315" t="n"/>
       <c r="M55" s="33" t="n"/>
-      <c r="N55" s="132" t="n"/>
-      <c r="O55" s="133" t="n"/>
+      <c r="N55" s="316" t="n"/>
+      <c r="O55" s="310" t="n"/>
       <c r="P55" s="34" t="n"/>
     </row>
     <row r="56" ht="21.9" customHeight="1">
@@ -4357,7 +4507,7 @@
     <row r="60" ht="21" customHeight="1">
       <c r="B60" s="74" t="n"/>
       <c r="C60" s="74" t="n"/>
-      <c r="D60" s="282" t="inlineStr">
+      <c r="D60" s="317" t="inlineStr">
         <is>
           <t>PROGRAMACIÓN DE FECHAS</t>
         </is>
@@ -4368,32 +4518,32 @@
     <row r="61" customFormat="1" s="123">
       <c r="B61" s="74" t="n"/>
       <c r="C61" s="74" t="n"/>
-      <c r="D61" s="283" t="inlineStr">
+      <c r="D61" s="318" t="inlineStr">
         <is>
           <t>ÁREA</t>
         </is>
       </c>
       <c r="E61" s="258" t="n"/>
       <c r="F61" s="259" t="n"/>
-      <c r="G61" s="284" t="inlineStr">
+      <c r="G61" s="319" t="inlineStr">
         <is>
           <t>INICIO</t>
         </is>
       </c>
       <c r="H61" s="191" t="n"/>
-      <c r="I61" s="285" t="inlineStr">
+      <c r="I61" s="320" t="inlineStr">
         <is>
           <t>TERMINA</t>
         </is>
       </c>
       <c r="J61" s="194" t="n"/>
-      <c r="K61" s="286" t="inlineStr">
-        <is>
-          <t>DIAS</t>
+      <c r="K61" s="321" t="inlineStr">
+        <is>
+          <t>DÍAS</t>
         </is>
       </c>
       <c r="L61" s="118" t="n"/>
-      <c r="M61" s="286" t="inlineStr">
+      <c r="M61" s="321" t="inlineStr">
         <is>
           <t>OBSERVACIONES</t>
         </is>
@@ -4436,16 +4586,16 @@
     <row r="63" ht="21" customHeight="1">
       <c r="B63" s="74" t="n"/>
       <c r="C63" s="74" t="n"/>
-      <c r="D63" s="276" t="n"/>
+      <c r="D63" s="322" t="n"/>
       <c r="E63" s="129" t="n"/>
       <c r="F63" s="130" t="n"/>
-      <c r="G63" s="210" t="n"/>
+      <c r="G63" s="323" t="n"/>
       <c r="H63" s="129" t="n"/>
-      <c r="I63" s="253" t="n"/>
+      <c r="I63" s="324" t="n"/>
       <c r="J63" s="196" t="n"/>
-      <c r="K63" s="253" t="n"/>
+      <c r="K63" s="324" t="n"/>
       <c r="L63" s="196" t="n"/>
-      <c r="M63" s="222" t="n"/>
+      <c r="M63" s="325" t="n"/>
       <c r="N63" s="129" t="n"/>
       <c r="O63" s="129" t="n"/>
       <c r="P63" s="130" t="n"/>
@@ -4480,16 +4630,16 @@
     <row r="65" ht="20.4" customFormat="1" customHeight="1" s="123">
       <c r="B65" s="74" t="n"/>
       <c r="C65" s="74" t="n"/>
-      <c r="D65" s="131" t="n"/>
+      <c r="D65" s="326" t="n"/>
       <c r="E65" s="129" t="n"/>
       <c r="F65" s="130" t="n"/>
-      <c r="G65" s="210" t="n"/>
+      <c r="G65" s="323" t="n"/>
       <c r="H65" s="129" t="n"/>
-      <c r="I65" s="253" t="n"/>
+      <c r="I65" s="324" t="n"/>
       <c r="J65" s="196" t="n"/>
-      <c r="K65" s="253" t="n"/>
+      <c r="K65" s="324" t="n"/>
       <c r="L65" s="196" t="n"/>
-      <c r="M65" s="222" t="n"/>
+      <c r="M65" s="325" t="n"/>
       <c r="N65" s="129" t="n"/>
       <c r="O65" s="129" t="n"/>
       <c r="P65" s="130" t="n"/>
@@ -4537,12 +4687,12 @@
     <row r="68" ht="24.9" customHeight="1">
       <c r="B68" s="74" t="n"/>
       <c r="C68" s="74" t="n"/>
-      <c r="D68" s="283" t="inlineStr">
+      <c r="D68" s="318" t="inlineStr">
         <is>
           <t>NO.</t>
         </is>
       </c>
-      <c r="E68" s="287" t="inlineStr">
+      <c r="E68" s="327" t="inlineStr">
         <is>
           <t>TRABAJOS PREVIOS A INICIAR</t>
         </is>
@@ -4589,10 +4739,10 @@
     <row r="70" ht="25.8" customHeight="1">
       <c r="B70" s="74" t="n"/>
       <c r="C70" s="74" t="n"/>
-      <c r="D70" s="110" t="n">
+      <c r="D70" s="328" t="n">
         <v>2</v>
       </c>
-      <c r="E70" s="303" t="n"/>
+      <c r="E70" s="329" t="n"/>
       <c r="F70" s="187" t="n"/>
       <c r="G70" s="187" t="n"/>
       <c r="H70" s="187" t="n"/>
@@ -4629,10 +4779,10 @@
     <row r="72" ht="24.9" customHeight="1">
       <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
-      <c r="D72" s="110" t="n">
+      <c r="D72" s="328" t="n">
         <v>4</v>
       </c>
-      <c r="E72" s="207" t="n"/>
+      <c r="E72" s="330" t="n"/>
       <c r="F72" s="129" t="n"/>
       <c r="G72" s="129" t="n"/>
       <c r="H72" s="129" t="n"/>
@@ -4684,14 +4834,14 @@
     <row r="75" ht="24.9" customHeight="1">
       <c r="B75" s="74" t="n"/>
       <c r="C75" s="74" t="n"/>
-      <c r="D75" s="298" t="inlineStr">
+      <c r="D75" s="331" t="inlineStr">
         <is>
           <t>NO.</t>
         </is>
       </c>
-      <c r="E75" s="299" t="inlineStr">
-        <is>
-          <t>SERVICIOS BASICOS NECESARIOS PARA TRABAJAR</t>
+      <c r="E75" s="332" t="inlineStr">
+        <is>
+          <t>SERVICIOS BÁSICOS NECESARIOS PARA TRABAJAR</t>
         </is>
       </c>
       <c r="F75" s="117" t="n"/>
@@ -4736,10 +4886,10 @@
     <row r="77" ht="24.9" customHeight="1">
       <c r="B77" s="74" t="n"/>
       <c r="C77" s="74" t="n"/>
-      <c r="D77" s="110" t="n">
+      <c r="D77" s="328" t="n">
         <v>2</v>
       </c>
-      <c r="E77" s="305" t="n"/>
+      <c r="E77" s="333" t="n"/>
       <c r="F77" s="187" t="n"/>
       <c r="G77" s="187" t="n"/>
       <c r="H77" s="187" t="n"/>
@@ -4778,10 +4928,10 @@
     <row r="79" ht="27" customHeight="1">
       <c r="B79" s="8" t="n"/>
       <c r="C79" s="8" t="n"/>
-      <c r="D79" s="110" t="n">
+      <c r="D79" s="328" t="n">
         <v>4</v>
       </c>
-      <c r="E79" s="254" t="n"/>
+      <c r="E79" s="334" t="n"/>
       <c r="F79" s="129" t="n"/>
       <c r="G79" s="129" t="n"/>
       <c r="H79" s="129" t="n"/>
@@ -4852,12 +5002,12 @@
     <row r="83" ht="24.9" customHeight="1">
       <c r="B83" s="8" t="n"/>
       <c r="C83" s="8" t="n"/>
-      <c r="D83" s="290" t="inlineStr">
+      <c r="D83" s="335" t="inlineStr">
         <is>
           <t>NO.</t>
         </is>
       </c>
-      <c r="E83" s="291" t="inlineStr">
+      <c r="E83" s="336" t="inlineStr">
         <is>
           <t>PUNTOS DE REVISIÓN ESPECÍFICA PARA RECEPCIÓN DE TRABAJOS</t>
         </is>
@@ -4893,10 +5043,10 @@
     <row r="85" ht="26.4" customHeight="1">
       <c r="B85" s="8" t="n"/>
       <c r="C85" s="8" t="n"/>
-      <c r="D85" s="155" t="n">
+      <c r="D85" s="337" t="n">
         <v>2</v>
       </c>
-      <c r="E85" s="301" t="n"/>
+      <c r="E85" s="338" t="n"/>
       <c r="F85" s="156" t="n"/>
       <c r="G85" s="156" t="n"/>
       <c r="H85" s="156" t="n"/>
@@ -4932,7 +5082,7 @@
       <c r="N86" s="4" t="n"/>
       <c r="O86" s="242" t="inlineStr">
         <is>
-          <t>Cartas firmadas por Lider de Proyecto y Maestro de obras, con fotografias de avance, cuadro de cantidades y renglones</t>
+          <t>Cartas firmadas por Líder de Proyecto y Maestro de obras, con fotografías de avance, cuadro de cantidades y renglones</t>
         </is>
       </c>
       <c r="Q86" s="44" t="n"/>
@@ -4946,10 +5096,10 @@
     <row r="87" ht="26.4" customHeight="1">
       <c r="B87" s="8" t="n"/>
       <c r="C87" s="8" t="n"/>
-      <c r="D87" s="155" t="n">
+      <c r="D87" s="337" t="n">
         <v>4</v>
       </c>
-      <c r="E87" s="134" t="n"/>
+      <c r="E87" s="339" t="n"/>
       <c r="F87" s="135" t="n"/>
       <c r="G87" s="135" t="n"/>
       <c r="H87" s="135" t="n"/>
@@ -4984,10 +5134,10 @@
     <row r="89" ht="27.6" customHeight="1">
       <c r="B89" s="8" t="n"/>
       <c r="C89" s="8" t="n"/>
-      <c r="D89" s="155" t="n">
+      <c r="D89" s="337" t="n">
         <v>6</v>
       </c>
-      <c r="E89" s="134" t="n"/>
+      <c r="E89" s="339" t="n"/>
       <c r="F89" s="135" t="n"/>
       <c r="G89" s="135" t="n"/>
       <c r="H89" s="135" t="n"/>
@@ -5026,10 +5176,10 @@
     <row r="91" ht="27.6" customHeight="1">
       <c r="B91" s="8" t="n"/>
       <c r="C91" s="8" t="n"/>
-      <c r="D91" s="155" t="n">
+      <c r="D91" s="337" t="n">
         <v>8</v>
       </c>
-      <c r="E91" s="134" t="n"/>
+      <c r="E91" s="339" t="n"/>
       <c r="F91" s="135" t="n"/>
       <c r="G91" s="135" t="n"/>
       <c r="H91" s="135" t="n"/>
@@ -5071,10 +5221,10 @@
     <row r="93" ht="27.6" customHeight="1">
       <c r="B93" s="8" t="n"/>
       <c r="C93" s="8" t="n"/>
-      <c r="D93" s="155" t="n">
+      <c r="D93" s="337" t="n">
         <v>10</v>
       </c>
-      <c r="E93" s="134" t="n"/>
+      <c r="E93" s="339" t="n"/>
       <c r="F93" s="135" t="n"/>
       <c r="G93" s="135" t="n"/>
       <c r="H93" s="135" t="n"/>
@@ -5086,7 +5236,7 @@
       <c r="N93" s="5" t="n"/>
       <c r="O93" s="242" t="inlineStr">
         <is>
-          <t>Contratista es el unico responsable de cumplir con los pagos directo a su personal en obra, tanto salario pactado como prestaciones en dado apliquen, quitando responsabilidad a E4 ante cualquier inconveniente</t>
+          <t>Contratista es el único responsable de cumplir con los pagos directo a su personal en obra, tanto salario pactado como prestaciones en dado caso apliquen, quitando responsabilidad a E4 ante cualquier inconveniente</t>
         </is>
       </c>
       <c r="Q93" s="44" t="n"/>
@@ -5114,10 +5264,10 @@
     <row r="95" ht="27.6" customHeight="1">
       <c r="B95" s="8" t="n"/>
       <c r="C95" s="8" t="n"/>
-      <c r="D95" s="155" t="n">
+      <c r="D95" s="337" t="n">
         <v>12</v>
       </c>
-      <c r="E95" s="134" t="n"/>
+      <c r="E95" s="339" t="n"/>
       <c r="F95" s="135" t="n"/>
       <c r="G95" s="135" t="n"/>
       <c r="H95" s="135" t="n"/>
@@ -5152,10 +5302,10 @@
     <row r="97" ht="27.6" customHeight="1">
       <c r="B97" s="8" t="n"/>
       <c r="C97" s="8" t="n"/>
-      <c r="D97" s="155" t="n">
+      <c r="D97" s="337" t="n">
         <v>14</v>
       </c>
-      <c r="E97" s="134" t="n"/>
+      <c r="E97" s="339" t="n"/>
       <c r="F97" s="135" t="n"/>
       <c r="G97" s="135" t="n"/>
       <c r="H97" s="135" t="n"/>
@@ -5194,10 +5344,10 @@
     <row r="99" ht="27.6" customHeight="1">
       <c r="B99" s="8" t="n"/>
       <c r="C99" s="8" t="n"/>
-      <c r="D99" s="155" t="n">
+      <c r="D99" s="337" t="n">
         <v>16</v>
       </c>
-      <c r="E99" s="134" t="n"/>
+      <c r="E99" s="339" t="n"/>
       <c r="F99" s="135" t="n"/>
       <c r="G99" s="135" t="n"/>
       <c r="H99" s="135" t="n"/>
@@ -5242,10 +5392,10 @@
     <row r="101" ht="27.6" customHeight="1">
       <c r="B101" s="8" t="n"/>
       <c r="C101" s="8" t="n"/>
-      <c r="D101" s="155" t="n">
+      <c r="D101" s="337" t="n">
         <v>18</v>
       </c>
-      <c r="E101" s="134" t="n"/>
+      <c r="E101" s="339" t="n"/>
       <c r="F101" s="135" t="n"/>
       <c r="G101" s="135" t="n"/>
       <c r="H101" s="135" t="n"/>
@@ -5280,10 +5430,10 @@
     <row r="103" ht="27.6" customHeight="1">
       <c r="B103" s="8" t="n"/>
       <c r="C103" s="8" t="n"/>
-      <c r="D103" s="155" t="n">
+      <c r="D103" s="337" t="n">
         <v>20</v>
       </c>
-      <c r="E103" s="134" t="n"/>
+      <c r="E103" s="339" t="n"/>
       <c r="F103" s="135" t="n"/>
       <c r="G103" s="135" t="n"/>
       <c r="H103" s="135" t="n"/>
@@ -5318,10 +5468,10 @@
     <row r="105" ht="27.6" customHeight="1">
       <c r="B105" s="8" t="n"/>
       <c r="C105" s="8" t="n"/>
-      <c r="D105" s="155" t="n">
+      <c r="D105" s="337" t="n">
         <v>22</v>
       </c>
-      <c r="E105" s="134" t="n"/>
+      <c r="E105" s="339" t="n"/>
       <c r="F105" s="135" t="n"/>
       <c r="G105" s="135" t="n"/>
       <c r="H105" s="135" t="n"/>
@@ -5360,10 +5510,10 @@
     <row r="107" ht="27.6" customHeight="1">
       <c r="B107" s="8" t="n"/>
       <c r="C107" s="8" t="n"/>
-      <c r="D107" s="155" t="n">
+      <c r="D107" s="337" t="n">
         <v>24</v>
       </c>
-      <c r="E107" s="134" t="n"/>
+      <c r="E107" s="339" t="n"/>
       <c r="F107" s="135" t="n"/>
       <c r="G107" s="135" t="n"/>
       <c r="H107" s="135" t="n"/>
@@ -5398,10 +5548,10 @@
     <row r="109" ht="27.6" customHeight="1">
       <c r="B109" s="8" t="n"/>
       <c r="C109" s="8" t="n"/>
-      <c r="D109" s="155" t="n">
+      <c r="D109" s="337" t="n">
         <v>26</v>
       </c>
-      <c r="E109" s="134" t="n"/>
+      <c r="E109" s="339" t="n"/>
       <c r="F109" s="135" t="n"/>
       <c r="G109" s="135" t="n"/>
       <c r="H109" s="135" t="n"/>
@@ -5436,10 +5586,10 @@
     <row r="111" ht="27.6" customHeight="1" thickBot="1">
       <c r="B111" s="8" t="n"/>
       <c r="C111" s="8" t="n"/>
-      <c r="D111" s="155" t="n">
+      <c r="D111" s="337" t="n">
         <v>28</v>
       </c>
-      <c r="E111" s="134" t="n"/>
+      <c r="E111" s="339" t="n"/>
       <c r="F111" s="135" t="n"/>
       <c r="G111" s="135" t="n"/>
       <c r="H111" s="135" t="n"/>
@@ -5499,9 +5649,9 @@
     <row r="114" ht="28.8" customHeight="1">
       <c r="B114" s="74" t="n"/>
       <c r="C114" s="74" t="n"/>
-      <c r="D114" s="214" t="inlineStr">
-        <is>
-          <t>AREA DE FIRMAS</t>
+      <c r="D114" s="340" t="inlineStr">
+        <is>
+          <t>ÁREA DE FIRMAS</t>
         </is>
       </c>
       <c r="Q114" s="55" t="n"/>
@@ -5736,12 +5886,207 @@
       <c r="Q125" s="55" t="n"/>
       <c r="R125" s="55" t="n"/>
     </row>
-    <row r="126">
+    <row r="126" ht="18" customHeight="1">
       <c r="Q126" s="55" t="n"/>
       <c r="R126" s="55" t="n"/>
     </row>
+    <row r="127" ht="24.9" customHeight="1">
+      <c r="B127" s="74" t="n"/>
+      <c r="C127" s="74" t="n"/>
+      <c r="D127" s="318" t="inlineStr">
+        <is>
+          <t>NO.</t>
+        </is>
+      </c>
+      <c r="E127" s="327" t="inlineStr">
+        <is>
+          <t>ANEXOS: DOCUMENTOS ADJUNTOS A LA SOLICITUD</t>
+        </is>
+      </c>
+      <c r="F127" s="117" t="n"/>
+      <c r="G127" s="117" t="n"/>
+      <c r="H127" s="117" t="n"/>
+      <c r="I127" s="117" t="n"/>
+      <c r="J127" s="117" t="n"/>
+      <c r="K127" s="117" t="n"/>
+      <c r="L127" s="117" t="n"/>
+      <c r="M127" s="117" t="n"/>
+      <c r="N127" s="117" t="n"/>
+      <c r="O127" s="117" t="n"/>
+      <c r="P127" s="118" t="n"/>
+      <c r="Q127" s="55" t="n"/>
+      <c r="R127" s="55" t="n"/>
+    </row>
+    <row r="128" ht="24.9" customHeight="1">
+      <c r="B128" s="74" t="n"/>
+      <c r="C128" s="99" t="n"/>
+      <c r="D128" s="108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" s="302" t="n"/>
+      <c r="F128" s="187" t="n"/>
+      <c r="G128" s="187" t="n"/>
+      <c r="H128" s="187" t="n"/>
+      <c r="I128" s="187" t="n"/>
+      <c r="J128" s="187" t="n"/>
+      <c r="K128" s="187" t="n"/>
+      <c r="L128" s="187" t="n"/>
+      <c r="M128" s="187" t="n"/>
+      <c r="N128" s="187" t="n"/>
+      <c r="O128" s="187" t="n"/>
+      <c r="P128" s="188" t="n"/>
+      <c r="Q128" s="99" t="n"/>
+      <c r="R128" s="99" t="n"/>
+    </row>
+    <row r="129" ht="25.8" customHeight="1">
+      <c r="B129" s="74" t="n"/>
+      <c r="C129" s="74" t="n"/>
+      <c r="D129" s="328" t="n">
+        <v>2</v>
+      </c>
+      <c r="E129" s="329" t="n"/>
+      <c r="F129" s="187" t="n"/>
+      <c r="G129" s="187" t="n"/>
+      <c r="H129" s="187" t="n"/>
+      <c r="I129" s="187" t="n"/>
+      <c r="J129" s="187" t="n"/>
+      <c r="K129" s="187" t="n"/>
+      <c r="L129" s="187" t="n"/>
+      <c r="M129" s="187" t="n"/>
+      <c r="N129" s="187" t="n"/>
+      <c r="O129" s="187" t="n"/>
+      <c r="P129" s="188" t="n"/>
+      <c r="Q129" s="55" t="n"/>
+      <c r="R129" s="55" t="n"/>
+    </row>
+    <row r="130" ht="24.9" customHeight="1">
+      <c r="B130" s="74" t="n"/>
+      <c r="C130" s="99" t="n"/>
+      <c r="D130" s="108" t="n">
+        <v>3</v>
+      </c>
+      <c r="E130" s="302" t="n"/>
+      <c r="F130" s="187" t="n"/>
+      <c r="G130" s="187" t="n"/>
+      <c r="H130" s="187" t="n"/>
+      <c r="I130" s="187" t="n"/>
+      <c r="J130" s="187" t="n"/>
+      <c r="K130" s="187" t="n"/>
+      <c r="L130" s="187" t="n"/>
+      <c r="M130" s="187" t="n"/>
+      <c r="N130" s="187" t="n"/>
+      <c r="O130" s="187" t="n"/>
+      <c r="P130" s="188" t="n"/>
+      <c r="Q130" s="99" t="n"/>
+      <c r="R130" s="99" t="n"/>
+    </row>
+    <row r="131" ht="25.8" customHeight="1">
+      <c r="B131" s="74" t="n"/>
+      <c r="C131" s="74" t="n"/>
+      <c r="D131" s="328" t="n">
+        <v>4</v>
+      </c>
+      <c r="E131" s="329" t="n"/>
+      <c r="F131" s="187" t="n"/>
+      <c r="G131" s="187" t="n"/>
+      <c r="H131" s="187" t="n"/>
+      <c r="I131" s="187" t="n"/>
+      <c r="J131" s="187" t="n"/>
+      <c r="K131" s="187" t="n"/>
+      <c r="L131" s="187" t="n"/>
+      <c r="M131" s="187" t="n"/>
+      <c r="N131" s="187" t="n"/>
+      <c r="O131" s="187" t="n"/>
+      <c r="P131" s="188" t="n"/>
+      <c r="Q131" s="55" t="n"/>
+      <c r="R131" s="55" t="n"/>
+    </row>
+    <row r="132" ht="24.9" customHeight="1">
+      <c r="B132" s="74" t="n"/>
+      <c r="C132" s="99" t="n"/>
+      <c r="D132" s="108" t="n">
+        <v>5</v>
+      </c>
+      <c r="E132" s="302" t="n"/>
+      <c r="F132" s="187" t="n"/>
+      <c r="G132" s="187" t="n"/>
+      <c r="H132" s="187" t="n"/>
+      <c r="I132" s="187" t="n"/>
+      <c r="J132" s="187" t="n"/>
+      <c r="K132" s="187" t="n"/>
+      <c r="L132" s="187" t="n"/>
+      <c r="M132" s="187" t="n"/>
+      <c r="N132" s="187" t="n"/>
+      <c r="O132" s="187" t="n"/>
+      <c r="P132" s="188" t="n"/>
+      <c r="Q132" s="99" t="n"/>
+      <c r="R132" s="99" t="n"/>
+    </row>
+    <row r="133" ht="25.8" customHeight="1">
+      <c r="B133" s="74" t="n"/>
+      <c r="C133" s="74" t="n"/>
+      <c r="D133" s="328" t="n">
+        <v>6</v>
+      </c>
+      <c r="E133" s="329" t="n"/>
+      <c r="F133" s="187" t="n"/>
+      <c r="G133" s="187" t="n"/>
+      <c r="H133" s="187" t="n"/>
+      <c r="I133" s="187" t="n"/>
+      <c r="J133" s="187" t="n"/>
+      <c r="K133" s="187" t="n"/>
+      <c r="L133" s="187" t="n"/>
+      <c r="M133" s="187" t="n"/>
+      <c r="N133" s="187" t="n"/>
+      <c r="O133" s="187" t="n"/>
+      <c r="P133" s="188" t="n"/>
+      <c r="Q133" s="55" t="n"/>
+      <c r="R133" s="55" t="n"/>
+    </row>
+    <row r="134" ht="24.9" customHeight="1">
+      <c r="B134" s="74" t="n"/>
+      <c r="C134" s="99" t="n"/>
+      <c r="D134" s="108" t="n">
+        <v>7</v>
+      </c>
+      <c r="E134" s="302" t="n"/>
+      <c r="F134" s="187" t="n"/>
+      <c r="G134" s="187" t="n"/>
+      <c r="H134" s="187" t="n"/>
+      <c r="I134" s="187" t="n"/>
+      <c r="J134" s="187" t="n"/>
+      <c r="K134" s="187" t="n"/>
+      <c r="L134" s="187" t="n"/>
+      <c r="M134" s="187" t="n"/>
+      <c r="N134" s="187" t="n"/>
+      <c r="O134" s="187" t="n"/>
+      <c r="P134" s="188" t="n"/>
+      <c r="Q134" s="99" t="n"/>
+      <c r="R134" s="99" t="n"/>
+    </row>
+    <row r="135" ht="25.8" customHeight="1">
+      <c r="B135" s="74" t="n"/>
+      <c r="C135" s="74" t="n"/>
+      <c r="D135" s="328" t="n">
+        <v>8</v>
+      </c>
+      <c r="E135" s="329" t="n"/>
+      <c r="F135" s="187" t="n"/>
+      <c r="G135" s="187" t="n"/>
+      <c r="H135" s="187" t="n"/>
+      <c r="I135" s="187" t="n"/>
+      <c r="J135" s="187" t="n"/>
+      <c r="K135" s="187" t="n"/>
+      <c r="L135" s="187" t="n"/>
+      <c r="M135" s="187" t="n"/>
+      <c r="N135" s="187" t="n"/>
+      <c r="O135" s="187" t="n"/>
+      <c r="P135" s="188" t="n"/>
+      <c r="Q135" s="55" t="n"/>
+      <c r="R135" s="55" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="198">
+  <mergeCells count="207">
     <mergeCell ref="M61:P61"/>
     <mergeCell ref="H123:J123"/>
     <mergeCell ref="D116:F116"/>
@@ -5785,6 +6130,7 @@
     <mergeCell ref="D45:I45"/>
     <mergeCell ref="D23:H23"/>
     <mergeCell ref="L38:O38"/>
+    <mergeCell ref="E135:P135"/>
     <mergeCell ref="E51:J51"/>
     <mergeCell ref="L31:O31"/>
     <mergeCell ref="L40:O40"/>
@@ -5802,6 +6148,7 @@
     <mergeCell ref="E77:P77"/>
     <mergeCell ref="E104:M104"/>
     <mergeCell ref="E49:J49"/>
+    <mergeCell ref="E133:P133"/>
     <mergeCell ref="E80:P80"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="K63:L63"/>
@@ -5816,6 +6163,7 @@
     <mergeCell ref="D33:I33"/>
     <mergeCell ref="D42:I42"/>
     <mergeCell ref="E72:P72"/>
+    <mergeCell ref="E134:P134"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="M64:P64"/>
     <mergeCell ref="G65:H65"/>
@@ -5891,17 +6239,21 @@
     <mergeCell ref="G63:H63"/>
     <mergeCell ref="K65:L65"/>
     <mergeCell ref="I63:J63"/>
+    <mergeCell ref="E127:P127"/>
     <mergeCell ref="D14:E14"/>
+    <mergeCell ref="E129:P129"/>
     <mergeCell ref="E88:M88"/>
     <mergeCell ref="L3:N3"/>
     <mergeCell ref="E79:P79"/>
     <mergeCell ref="L25:O25"/>
     <mergeCell ref="E73:P73"/>
     <mergeCell ref="I65:J65"/>
+    <mergeCell ref="E131:P131"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D18:J18"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="F16:J16"/>
+    <mergeCell ref="E128:P128"/>
     <mergeCell ref="O116:P116"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="M66:P66"/>
@@ -5930,6 +6282,7 @@
     <mergeCell ref="F13:J13"/>
     <mergeCell ref="L15:O15"/>
     <mergeCell ref="D63:F63"/>
+    <mergeCell ref="E130:P130"/>
     <mergeCell ref="E68:P68"/>
     <mergeCell ref="O122:P122"/>
     <mergeCell ref="D46:I46"/>
@@ -5937,6 +6290,7 @@
     <mergeCell ref="E111:M111"/>
     <mergeCell ref="D40:I40"/>
     <mergeCell ref="D65:F65"/>
+    <mergeCell ref="E132:P132"/>
     <mergeCell ref="N49:O49"/>
     <mergeCell ref="K62:L62"/>
     <mergeCell ref="E87:M87"/>

</xml_diff>